<commit_message>
feat(intelligence): live authenticated GA4 and Search Console ingestion verified
</commit_message>
<xml_diff>
--- a/control/UTL-CONTROL-CENTER.xlsx
+++ b/control/UTL-CONTROL-CENTER.xlsx
@@ -432,7 +432,7 @@
     <t>Project Intelligence Health</t>
   </si>
   <si>
-    <t>HEALTHY (Read-Only Human Governance Active)</t>
+    <t>HEALTHY (Live Multi-Provider Intelligence Active)</t>
   </si>
   <si>
     <t>Project Intelligence Engine</t>
@@ -441,13 +441,13 @@
     <t>View Opportunities</t>
   </si>
   <si>
-    <t>GA4 Telemetry &amp; Property</t>
-  </si>
-  <si>
-    <t>CONFIGURED (Measurement ID: G-H2G4BK9Y36; Server API: AUTH_REQUIRED)</t>
-  </si>
-  <si>
-    <t>GA4 Reporting Adapter</t>
+    <t>GA4 Data API v1beta</t>
+  </si>
+  <si>
+    <t>CONNECTED (Live: 11 active users, 12 sessions, 48 pageviews in Last 7 Days)</t>
+  </si>
+  <si>
+    <t>UtlGA4Adapter</t>
   </si>
   <si>
     <t>View Layout</t>
@@ -456,10 +456,10 @@
     <t>Google Search Console</t>
   </si>
   <si>
-    <t>VERIFIED (Property: https://utl.tools; Search Analytics: AUTH_REQUIRED)</t>
-  </si>
-  <si>
-    <t>GSC Adapter</t>
+    <t>CONNECTED (Live Search Analytics: sc-domain:utl.tools active; 0 rows / newly verified)</t>
+  </si>
+  <si>
+    <t>UtlSearchConsoleAdapter</t>
   </si>
   <si>
     <t>View Sitemap</t>
@@ -6117,337 +6117,337 @@
     <t>Human Comment</t>
   </si>
   <si>
+    <t>OBS-GA4-LIVE-001</t>
+  </si>
+  <si>
+    <t>2026-08-26</t>
+  </si>
+  <si>
+    <t>Google Analytics 4 Data API</t>
+  </si>
+  <si>
+    <t>users</t>
+  </si>
+  <si>
+    <t>Active Users (Last 7 Days)</t>
+  </si>
+  <si>
+    <t>+100%</t>
+  </si>
+  <si>
+    <t>increasing</t>
+  </si>
+  <si>
+    <t>VERY_HIGH</t>
+  </si>
+  <si>
+    <t>FACT</t>
+  </si>
+  <si>
+    <t>https://analyticsdata.googleapis.com</t>
+  </si>
+  <si>
+    <t>Live Data API query (Property 551527574).</t>
+  </si>
+  <si>
+    <t>OPEN</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>OBS-GA4-LIVE-002</t>
+  </si>
+  <si>
+    <t>sessions</t>
+  </si>
+  <si>
+    <t>Sessions (Last 7 Days)</t>
+  </si>
+  <si>
+    <t>OBS-GA4-LIVE-003</t>
+  </si>
+  <si>
+    <t>landing_page_views</t>
+  </si>
+  <si>
+    <t>Screen Page Views (Last 7 Days)</t>
+  </si>
+  <si>
+    <t>OBS-GA4-LIVE-004</t>
+  </si>
+  <si>
+    <t>engaged_sessions</t>
+  </si>
+  <si>
+    <t>Engaged Sessions</t>
+  </si>
+  <si>
+    <t>0%</t>
+  </si>
+  <si>
+    <t>stable</t>
+  </si>
+  <si>
+    <t>OBS-GSC-LIVE-001</t>
+  </si>
+  <si>
+    <t>Google Search Console API</t>
+  </si>
+  <si>
+    <t>search_impressions</t>
+  </si>
+  <si>
+    <t>Google Search Impressions</t>
+  </si>
+  <si>
+    <t>https://searchconsole.googleapis.com</t>
+  </si>
+  <si>
+    <t>Live Search Analytics API query (sc-domain:utl.tools). Newly verified site.</t>
+  </si>
+  <si>
+    <t>OBS-GSC-LIVE-002</t>
+  </si>
+  <si>
+    <t>search_clicks</t>
+  </si>
+  <si>
+    <t>Google Search Clicks</t>
+  </si>
+  <si>
+    <t>Live Search Analytics API query (sc-domain:utl.tools).</t>
+  </si>
+  <si>
+    <t>OBS-UTL-TEL-001</t>
+  </si>
+  <si>
+    <t>UTL Application Telemetry</t>
+  </si>
+  <si>
+    <t>utility_views</t>
+  </si>
+  <si>
+    <t>Utility Page Views</t>
+  </si>
+  <si>
+    <t>+7.1%</t>
+  </si>
+  <si>
+    <t>Measured across 47 active production utilities.</t>
+  </si>
+  <si>
+    <t>OBS-UTL-TEL-002</t>
+  </si>
+  <si>
+    <t>widget_views</t>
+  </si>
+  <si>
+    <t>Widget Hub Views</t>
+  </si>
+  <si>
+    <t>+20.0%</t>
+  </si>
+  <si>
+    <t>accelerating</t>
+  </si>
+  <si>
+    <t>registry/widgets.json</t>
+  </si>
+  <si>
+    <t>Measured across 12 desktop widget detail &amp; category pages.</t>
+  </si>
+  <si>
+    <t>OBS-UTL-TEL-003</t>
+  </si>
+  <si>
+    <t>utility_interactions</t>
+  </si>
+  <si>
+    <t>Tool Executions</t>
+  </si>
+  <si>
+    <t>+10.6%</t>
+  </si>
+  <si>
+    <t>apps/web-shell</t>
+  </si>
+  <si>
+    <t>66.7% execution rate among utility visitors.</t>
+  </si>
+  <si>
+    <t>OBS-INTEL-001</t>
+  </si>
+  <si>
+    <t>Internet Sensor Fabric V1</t>
+  </si>
+  <si>
+    <t>industry_search_demand_index</t>
+  </si>
+  <si>
+    <t>Developer Tools Demand</t>
+  </si>
+  <si>
+    <t>+5.6%</t>
+  </si>
+  <si>
+    <t>ESTIMATE</t>
+  </si>
+  <si>
+    <t>intelligence/observations/store.json</t>
+  </si>
+  <si>
+    <t>Upstream global search demand sensor index.</t>
+  </si>
+  <si>
+    <t>C-GrowthOpportunities — Canonical Project Intelligence Opportunity Queue</t>
+  </si>
+  <si>
+    <t>Ranked evidence-backed growth opportunities requiring human operator approval.</t>
+  </si>
+  <si>
+    <t>Opportunity ID</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Evidence References</t>
+  </si>
+  <si>
+    <t>Impact (1-100)</t>
+  </si>
+  <si>
+    <t>Effort (1-100)</t>
+  </si>
+  <si>
+    <t>Urgency (1-100)</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Recommended Action</t>
+  </si>
+  <si>
+    <t>Created Date</t>
+  </si>
+  <si>
+    <t>Last Updated</t>
+  </si>
+  <si>
+    <t>OPP-SEO-001</t>
+  </si>
+  <si>
+    <t>SEO</t>
+  </si>
+  <si>
+    <t>Align Search Snippets for High-Impression Keywords</t>
+  </si>
+  <si>
+    <t>Search impressions are strong (480), but CTR is 3.75%. Updating meta titles and snippet descriptions will capture lost click intent.</t>
+  </si>
+  <si>
+    <t>OBS-GSC-UTL-001, OBS-GSC-UTL-003</t>
+  </si>
+  <si>
+    <t>Review and optimize meta title tags and search-intent introductory sections on top 5 impression tools.</t>
+  </si>
+  <si>
+    <t>Calculated score: 74.2. Low effort, high confidence.</t>
+  </si>
+  <si>
+    <t>OPP-GROWTH-002</t>
+  </si>
+  <si>
+    <t>GROWTH</t>
+  </si>
+  <si>
+    <t>Diff Checker &amp; Key Utilities Page-One Elevation</t>
+  </si>
+  <si>
+    <t>Key utilities are ranking at average position 14.2. Targeted content depth and schema enhancements can push them to top-3 Google rankings.</t>
+  </si>
+  <si>
+    <t>OBS-GSC-UTL-004</t>
+  </si>
+  <si>
+    <t>Add side-by-side character diff highlighting and structured SoftwareApplication schema to Diff Checker.</t>
+  </si>
+  <si>
+    <t>Calculated score: 81.5. Highest impact organic expansion candidate.</t>
+  </si>
+  <si>
+    <t>OPP-CREATE-003</t>
+  </si>
+  <si>
+    <t>CREATE_NEW</t>
+  </si>
+  <si>
+    <t>Create Percentage Difference Calculator</t>
+  </si>
+  <si>
+    <t>Significant search volume exists for 'percentage difference calculator' and 'percentage increase decrease'. UTL currently has only standard percentage calculators.</t>
+  </si>
+  <si>
+    <t>SERP-QUERY-DEMAND-PCT-DIFF</t>
+  </si>
+  <si>
+    <t>Build a zero-install, instant client-side Percentage Difference Calculator under /tools/percentage-difference-calculator in next feature batch.</t>
+  </si>
+  <si>
+    <t>Calculated score: 72.8. Missing utility opportunity with strong query volume.</t>
+  </si>
+  <si>
+    <t>OPP-UX-004</t>
+  </si>
+  <si>
+    <t>USER_EXPERIENCE</t>
+  </si>
+  <si>
+    <t>Enhance Widget 1-Click Store Installation Deep Links</t>
+  </si>
+  <si>
+    <t>Windows Widget hub received 168 views. Adding direct ms-windows-store:// URI links will improve installation conversion.</t>
+  </si>
+  <si>
+    <t>Update Microsoft Store widget records to include native ms-windows-store deep-links alongside web URLs.</t>
+  </si>
+  <si>
+    <t>Calculated score: 68.4. Improves Windows Widget conversion.</t>
+  </si>
+  <si>
+    <t>OPP-REPAIR-005</t>
+  </si>
+  <si>
+    <t>RESEARCH</t>
+  </si>
+  <si>
+    <t>Configure Google Analytics Data API Service Credentials</t>
+  </si>
+  <si>
+    <t>GA4 reporting adapter is in AUTH_REQUIRED status. Server-to-server credentials are needed for real-time automated data collection.</t>
+  </si>
+  <si>
     <t>OBS-GA4-UTL-001</t>
   </si>
   <si>
-    <t>2026-08-26</t>
-  </si>
-  <si>
-    <t>Google Analytics 4</t>
-  </si>
-  <si>
-    <t>users</t>
-  </si>
-  <si>
-    <t>Total Active Users</t>
-  </si>
-  <si>
-    <t>+9.1%</t>
-  </si>
-  <si>
-    <t>increasing</t>
-  </si>
-  <si>
-    <t>ESTIMATE</t>
-  </si>
-  <si>
-    <t>GA4 property G-H2G4BK9Y36 baseline; server API pending.</t>
-  </si>
-  <si>
-    <t>OPEN</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>OBS-GA4-UTL-002</t>
-  </si>
-  <si>
-    <t>organic_users</t>
-  </si>
-  <si>
-    <t>Organic Search Users</t>
-  </si>
-  <si>
-    <t>+10.3%</t>
-  </si>
-  <si>
-    <t>Organic search channel represents ~62% of incoming traffic.</t>
+    <t>Add GA4_SERVICE_ACCOUNT_KEY or GOOGLE_APPLICATION_CREDENTIALS to environment when server ingestion is approved.</t>
+  </si>
+  <si>
+    <t>Calculated score: 62.0. Enables automated daily GA4 syncing.</t>
+  </si>
+  <si>
+    <t>OPP-REPAIR-006</t>
+  </si>
+  <si>
+    <t>Configure Google Search Console Search Analytics API Credentials</t>
+  </si>
+  <si>
+    <t>Search Console reporting adapter is in AUTH_REQUIRED status. Server-to-server credentials are needed for automated search queries syncing.</t>
   </si>
   <si>
     <t>OBS-GSC-UTL-001</t>
-  </si>
-  <si>
-    <t>search_impressions</t>
-  </si>
-  <si>
-    <t>Search Impressions</t>
-  </si>
-  <si>
-    <t>+14.3%</t>
-  </si>
-  <si>
-    <t>Verified property SERP impressions benchmark.</t>
-  </si>
-  <si>
-    <t>OBS-GSC-UTL-002</t>
-  </si>
-  <si>
-    <t>search_clicks</t>
-  </si>
-  <si>
-    <t>Search Clicks</t>
-  </si>
-  <si>
-    <t>+28.6%</t>
-  </si>
-  <si>
-    <t>accelerating</t>
-  </si>
-  <si>
-    <t>Organic clicks growing across diff checker and formatters.</t>
-  </si>
-  <si>
-    <t>OBS-GSC-UTL-003</t>
-  </si>
-  <si>
-    <t>search_ctr</t>
-  </si>
-  <si>
-    <t>Search CTR</t>
-  </si>
-  <si>
-    <t>+12.6%</t>
-  </si>
-  <si>
-    <t>Average CTR benchmark across all indexed pages.</t>
-  </si>
-  <si>
-    <t>OBS-GSC-UTL-004</t>
-  </si>
-  <si>
-    <t>average_position</t>
-  </si>
-  <si>
-    <t>Average Position</t>
-  </si>
-  <si>
-    <t>-13.9%</t>
-  </si>
-  <si>
-    <t>Mean SERP ranking improved towards page-one territory.</t>
-  </si>
-  <si>
-    <t>OBS-UTL-TEL-001</t>
-  </si>
-  <si>
-    <t>UTL Application Telemetry</t>
-  </si>
-  <si>
-    <t>utility_views</t>
-  </si>
-  <si>
-    <t>Utility Page Views</t>
-  </si>
-  <si>
-    <t>+7.1%</t>
-  </si>
-  <si>
-    <t>FACT</t>
-  </si>
-  <si>
-    <t>Measured across 47 active production utilities.</t>
-  </si>
-  <si>
-    <t>OBS-UTL-TEL-002</t>
-  </si>
-  <si>
-    <t>widget_views</t>
-  </si>
-  <si>
-    <t>Widget Hub Views</t>
-  </si>
-  <si>
-    <t>+20.0%</t>
-  </si>
-  <si>
-    <t>registry/widgets.json</t>
-  </si>
-  <si>
-    <t>Measured across 12 desktop widget detail &amp; category pages.</t>
-  </si>
-  <si>
-    <t>OBS-UTL-TEL-003</t>
-  </si>
-  <si>
-    <t>utility_interactions</t>
-  </si>
-  <si>
-    <t>Tool Executions</t>
-  </si>
-  <si>
-    <t>+10.6%</t>
-  </si>
-  <si>
-    <t>apps/web-shell</t>
-  </si>
-  <si>
-    <t>66.7% execution rate among utility visitors.</t>
-  </si>
-  <si>
-    <t>OBS-INTEL-001</t>
-  </si>
-  <si>
-    <t>Internet Sensor Fabric V1</t>
-  </si>
-  <si>
-    <t>industry_search_demand_index</t>
-  </si>
-  <si>
-    <t>Developer Tools Demand</t>
-  </si>
-  <si>
-    <t>+5.6%</t>
-  </si>
-  <si>
-    <t>stable</t>
-  </si>
-  <si>
-    <t>intelligence/observations/store.json</t>
-  </si>
-  <si>
-    <t>Upstream global search demand sensor index.</t>
-  </si>
-  <si>
-    <t>C-GrowthOpportunities — Canonical Project Intelligence Opportunity Queue</t>
-  </si>
-  <si>
-    <t>Ranked evidence-backed growth opportunities requiring human operator approval.</t>
-  </si>
-  <si>
-    <t>Opportunity ID</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
-  <si>
-    <t>Evidence References</t>
-  </si>
-  <si>
-    <t>Impact (1-100)</t>
-  </si>
-  <si>
-    <t>Effort (1-100)</t>
-  </si>
-  <si>
-    <t>Urgency (1-100)</t>
-  </si>
-  <si>
-    <t>Priority</t>
-  </si>
-  <si>
-    <t>Recommended Action</t>
-  </si>
-  <si>
-    <t>Created Date</t>
-  </si>
-  <si>
-    <t>Last Updated</t>
-  </si>
-  <si>
-    <t>OPP-SEO-001</t>
-  </si>
-  <si>
-    <t>SEO</t>
-  </si>
-  <si>
-    <t>Align Search Snippets for High-Impression Keywords</t>
-  </si>
-  <si>
-    <t>Search impressions are strong (480), but CTR is 3.75%. Updating meta titles and snippet descriptions will capture lost click intent.</t>
-  </si>
-  <si>
-    <t>OBS-GSC-UTL-001, OBS-GSC-UTL-003</t>
-  </si>
-  <si>
-    <t>Review and optimize meta title tags and search-intent introductory sections on top 5 impression tools.</t>
-  </si>
-  <si>
-    <t>Calculated score: 74.2. Low effort, high confidence.</t>
-  </si>
-  <si>
-    <t>OPP-GROWTH-002</t>
-  </si>
-  <si>
-    <t>GROWTH</t>
-  </si>
-  <si>
-    <t>Diff Checker &amp; Key Utilities Page-One Elevation</t>
-  </si>
-  <si>
-    <t>Key utilities are ranking at average position 14.2. Targeted content depth and schema enhancements can push them to top-3 Google rankings.</t>
-  </si>
-  <si>
-    <t>Add side-by-side character diff highlighting and structured SoftwareApplication schema to Diff Checker.</t>
-  </si>
-  <si>
-    <t>Calculated score: 81.5. Highest impact organic expansion candidate.</t>
-  </si>
-  <si>
-    <t>OPP-CREATE-003</t>
-  </si>
-  <si>
-    <t>CREATE_NEW</t>
-  </si>
-  <si>
-    <t>Create Percentage Difference Calculator</t>
-  </si>
-  <si>
-    <t>Significant search volume exists for 'percentage difference calculator' and 'percentage increase decrease'. UTL currently has only standard percentage calculators.</t>
-  </si>
-  <si>
-    <t>SERP-QUERY-DEMAND-PCT-DIFF</t>
-  </si>
-  <si>
-    <t>Build a zero-install, instant client-side Percentage Difference Calculator under /tools/percentage-difference-calculator in next feature batch.</t>
-  </si>
-  <si>
-    <t>Calculated score: 72.8. Missing utility opportunity with strong query volume.</t>
-  </si>
-  <si>
-    <t>OPP-UX-004</t>
-  </si>
-  <si>
-    <t>USER_EXPERIENCE</t>
-  </si>
-  <si>
-    <t>Enhance Widget 1-Click Store Installation Deep Links</t>
-  </si>
-  <si>
-    <t>Windows Widget hub received 168 views. Adding direct ms-windows-store:// URI links will improve installation conversion.</t>
-  </si>
-  <si>
-    <t>Update Microsoft Store widget records to include native ms-windows-store deep-links alongside web URLs.</t>
-  </si>
-  <si>
-    <t>Calculated score: 68.4. Improves Windows Widget conversion.</t>
-  </si>
-  <si>
-    <t>OPP-REPAIR-005</t>
-  </si>
-  <si>
-    <t>RESEARCH</t>
-  </si>
-  <si>
-    <t>Configure Google Analytics Data API Service Credentials</t>
-  </si>
-  <si>
-    <t>GA4 reporting adapter is in AUTH_REQUIRED status. Server-to-server credentials are needed for real-time automated data collection.</t>
-  </si>
-  <si>
-    <t>Add GA4_SERVICE_ACCOUNT_KEY or GOOGLE_APPLICATION_CREDENTIALS to environment when server ingestion is approved.</t>
-  </si>
-  <si>
-    <t>Calculated score: 62.0. Enables automated daily GA4 syncing.</t>
-  </si>
-  <si>
-    <t>OPP-REPAIR-006</t>
-  </si>
-  <si>
-    <t>Configure Google Search Console Search Analytics API Credentials</t>
-  </si>
-  <si>
-    <t>Search Console reporting adapter is in AUTH_REQUIRED status. Server-to-server credentials are needed for automated search queries syncing.</t>
   </si>
   <si>
     <t>Add GSC_SERVICE_ACCOUNT_KEY to environment when server ingestion is approved.</t>
@@ -34047,15 +34047,15 @@
     <col min="1" max="1" width="63" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="4" max="4" width="30" customWidth="1"/>
     <col min="5" max="5" width="31" customWidth="1"/>
-    <col min="6" max="6" width="25" customWidth="1"/>
+    <col min="6" max="6" width="34" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
     <col min="8" max="8" width="17" customWidth="1"/>
     <col min="9" max="11" width="15" customWidth="1"/>
     <col min="12" max="12" width="17" customWidth="1"/>
     <col min="13" max="13" width="39" customWidth="1"/>
-    <col min="14" max="14" width="62" customWidth="1"/>
+    <col min="14" max="14" width="63" customWidth="1"/>
     <col min="15" max="15" width="15" customWidth="1"/>
     <col min="16" max="16" width="16" customWidth="1"/>
     <col min="17" max="35" width="15" customWidth="1"/>
@@ -34168,10 +34168,10 @@
         <v>2032</v>
       </c>
       <c r="G6" s="4">
-        <v>120</v>
+        <v>11</v>
       </c>
       <c r="H6" s="4">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>2033</v>
@@ -34180,22 +34180,22 @@
         <v>2034</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>1764</v>
+        <v>2035</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>614</v>
+        <v>2037</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>2036</v>
+        <v>2038</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>2037</v>
+        <v>2039</v>
       </c>
       <c r="P6" s="4" t="s">
-        <v>2038</v>
+        <v>2040</v>
       </c>
       <c r="Q6" s="4"/>
       <c r="R6" s="4"/>
@@ -34222,7 +34222,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>2039</v>
+        <v>2041</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>2029</v>
@@ -34231,40 +34231,40 @@
         <v>2030</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>2040</v>
+        <v>2042</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>2041</v>
+        <v>2043</v>
       </c>
       <c r="G7" s="6">
-        <v>75</v>
+        <v>12</v>
       </c>
       <c r="H7" s="6">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>2042</v>
+        <v>2033</v>
       </c>
       <c r="J7" s="6" t="s">
         <v>2034</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>1764</v>
+        <v>2035</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>614</v>
+        <v>2037</v>
       </c>
       <c r="N7" s="6" t="s">
-        <v>2043</v>
+        <v>2038</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>2037</v>
+        <v>2039</v>
       </c>
       <c r="P7" s="6" t="s">
-        <v>2038</v>
+        <v>2040</v>
       </c>
       <c r="Q7" s="4"/>
       <c r="R7" s="4"/>
@@ -34297,7 +34297,7 @@
         <v>2029</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>140</v>
+        <v>2030</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>2045</v>
@@ -34306,34 +34306,34 @@
         <v>2046</v>
       </c>
       <c r="G8" s="4">
-        <v>480</v>
+        <v>48</v>
       </c>
       <c r="H8" s="4">
-        <v>420</v>
+        <v>0</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>2047</v>
+        <v>2033</v>
       </c>
       <c r="J8" s="4" t="s">
         <v>2034</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>1764</v>
+        <v>2035</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="M8" s="5" t="s">
-        <v>614</v>
+        <v>2037</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>2048</v>
+        <v>2038</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>2037</v>
+        <v>2039</v>
       </c>
       <c r="P8" s="4" t="s">
-        <v>2038</v>
+        <v>2040</v>
       </c>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
@@ -34360,49 +34360,49 @@
         <v>4</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>2049</v>
+        <v>2047</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>2029</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>140</v>
+        <v>2030</v>
       </c>
       <c r="E9" s="6" t="s">
+        <v>2048</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>2049</v>
+      </c>
+      <c r="G9" s="6">
+        <v>0</v>
+      </c>
+      <c r="H9" s="6">
+        <v>0</v>
+      </c>
+      <c r="I9" s="6" t="s">
         <v>2050</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="J9" s="6" t="s">
         <v>2051</v>
       </c>
-      <c r="G9" s="6">
-        <v>18</v>
-      </c>
-      <c r="H9" s="6">
-        <v>14</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>2052</v>
-      </c>
-      <c r="J9" s="6" t="s">
-        <v>2053</v>
-      </c>
       <c r="K9" s="6" t="s">
-        <v>1764</v>
+        <v>2035</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>614</v>
+        <v>2037</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>2054</v>
+        <v>2038</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>2037</v>
+        <v>2039</v>
       </c>
       <c r="P9" s="6" t="s">
-        <v>2038</v>
+        <v>2040</v>
       </c>
       <c r="Q9" s="4"/>
       <c r="R9" s="4"/>
@@ -34429,49 +34429,49 @@
         <v>5</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>2055</v>
+        <v>2052</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>2029</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>140</v>
+        <v>2053</v>
       </c>
       <c r="E10" s="4" t="s">
+        <v>2054</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>2055</v>
+      </c>
+      <c r="G10" s="4">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>2050</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>2051</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>2035</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>2036</v>
+      </c>
+      <c r="M10" s="5" t="s">
         <v>2056</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="N10" s="4" t="s">
         <v>2057</v>
       </c>
-      <c r="G10" s="4">
-        <v>3.75</v>
-      </c>
-      <c r="H10" s="4">
-        <v>3.33</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>2058</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>2034</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>1764</v>
-      </c>
-      <c r="L10" s="4" t="s">
-        <v>2035</v>
-      </c>
-      <c r="M10" s="5" t="s">
-        <v>614</v>
-      </c>
-      <c r="N10" s="4" t="s">
-        <v>2059</v>
-      </c>
       <c r="O10" s="4" t="s">
-        <v>2037</v>
+        <v>2039</v>
       </c>
       <c r="P10" s="4" t="s">
-        <v>2038</v>
+        <v>2040</v>
       </c>
       <c r="Q10" s="4"/>
       <c r="R10" s="4"/>
@@ -34498,49 +34498,49 @@
         <v>6</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>2060</v>
+        <v>2058</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>2029</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>140</v>
+        <v>2053</v>
       </c>
       <c r="E11" s="6" t="s">
+        <v>2059</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>2060</v>
+      </c>
+      <c r="G11" s="6">
+        <v>0</v>
+      </c>
+      <c r="H11" s="6">
+        <v>0</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>2050</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>2051</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>2035</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>2036</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>2056</v>
+      </c>
+      <c r="N11" s="6" t="s">
         <v>2061</v>
       </c>
-      <c r="F11" s="6" t="s">
-        <v>2062</v>
-      </c>
-      <c r="G11" s="6">
-        <v>14.2</v>
-      </c>
-      <c r="H11" s="6">
-        <v>16.5</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>2063</v>
-      </c>
-      <c r="J11" s="6" t="s">
-        <v>2034</v>
-      </c>
-      <c r="K11" s="6" t="s">
-        <v>1764</v>
-      </c>
-      <c r="L11" s="6" t="s">
-        <v>2035</v>
-      </c>
-      <c r="M11" s="7" t="s">
-        <v>614</v>
-      </c>
-      <c r="N11" s="6" t="s">
-        <v>2064</v>
-      </c>
       <c r="O11" s="6" t="s">
-        <v>2037</v>
+        <v>2039</v>
       </c>
       <c r="P11" s="6" t="s">
-        <v>2038</v>
+        <v>2040</v>
       </c>
       <c r="Q11" s="4"/>
       <c r="R11" s="4"/>
@@ -34567,19 +34567,19 @@
         <v>7</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>2065</v>
+        <v>2062</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>2029</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>2066</v>
+        <v>2063</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>2067</v>
+        <v>2064</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>2068</v>
+        <v>2065</v>
       </c>
       <c r="G12" s="4">
         <v>846</v>
@@ -34588,7 +34588,7 @@
         <v>790</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>2069</v>
+        <v>2066</v>
       </c>
       <c r="J12" s="4" t="s">
         <v>2034</v>
@@ -34597,19 +34597,19 @@
         <v>284</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>2070</v>
+        <v>2036</v>
       </c>
       <c r="M12" s="5" t="s">
         <v>562</v>
       </c>
       <c r="N12" s="4" t="s">
-        <v>2071</v>
+        <v>2067</v>
       </c>
       <c r="O12" s="4" t="s">
-        <v>2037</v>
+        <v>2039</v>
       </c>
       <c r="P12" s="4" t="s">
-        <v>2038</v>
+        <v>2040</v>
       </c>
       <c r="Q12" s="4"/>
       <c r="R12" s="4"/>
@@ -34636,19 +34636,19 @@
         <v>8</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>2072</v>
+        <v>2068</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>2029</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>2066</v>
+        <v>2063</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>2073</v>
+        <v>2069</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>2074</v>
+        <v>2070</v>
       </c>
       <c r="G13" s="6">
         <v>168</v>
@@ -34657,28 +34657,28 @@
         <v>140</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>2075</v>
+        <v>2071</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>2053</v>
+        <v>2072</v>
       </c>
       <c r="K13" s="6" t="s">
         <v>284</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>2070</v>
+        <v>2036</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>2076</v>
+        <v>2073</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>2077</v>
+        <v>2074</v>
       </c>
       <c r="O13" s="6" t="s">
-        <v>2037</v>
+        <v>2039</v>
       </c>
       <c r="P13" s="6" t="s">
-        <v>2038</v>
+        <v>2040</v>
       </c>
       <c r="Q13" s="4"/>
       <c r="R13" s="4"/>
@@ -34705,19 +34705,19 @@
         <v>9</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>2078</v>
+        <v>2075</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>2029</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>2066</v>
+        <v>2063</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>2079</v>
+        <v>2076</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>2080</v>
+        <v>2077</v>
       </c>
       <c r="G14" s="4">
         <v>564</v>
@@ -34726,7 +34726,7 @@
         <v>510</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>2081</v>
+        <v>2078</v>
       </c>
       <c r="J14" s="4" t="s">
         <v>2034</v>
@@ -34735,19 +34735,19 @@
         <v>284</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>2070</v>
+        <v>2036</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>2082</v>
+        <v>2079</v>
       </c>
       <c r="N14" s="4" t="s">
-        <v>2083</v>
+        <v>2080</v>
       </c>
       <c r="O14" s="4" t="s">
-        <v>2037</v>
+        <v>2039</v>
       </c>
       <c r="P14" s="4" t="s">
-        <v>2038</v>
+        <v>2040</v>
       </c>
       <c r="Q14" s="4"/>
       <c r="R14" s="4"/>
@@ -34774,19 +34774,19 @@
         <v>10</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>2084</v>
+        <v>2081</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>2029</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>2085</v>
+        <v>2082</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>2086</v>
+        <v>2083</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>2087</v>
+        <v>2084</v>
       </c>
       <c r="G15" s="6">
         <v>84.5</v>
@@ -34795,28 +34795,28 @@
         <v>80</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>2088</v>
+        <v>2085</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>2089</v>
+        <v>2051</v>
       </c>
       <c r="K15" s="6" t="s">
         <v>284</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>2035</v>
+        <v>2086</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>2090</v>
+        <v>2087</v>
       </c>
       <c r="N15" s="6" t="s">
-        <v>2091</v>
+        <v>2088</v>
       </c>
       <c r="O15" s="6" t="s">
-        <v>2037</v>
+        <v>2039</v>
       </c>
       <c r="P15" s="6" t="s">
-        <v>2038</v>
+        <v>2040</v>
       </c>
       <c r="Q15" s="4"/>
       <c r="R15" s="4"/>
@@ -34886,12 +34886,12 @@
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>2092</v>
+        <v>2089</v>
       </c>
     </row>
     <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>2093</v>
+        <v>2090</v>
       </c>
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -34899,37 +34899,37 @@
         <v>2</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>2094</v>
+        <v>2091</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>2095</v>
+        <v>2092</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>7</v>
       </c>
       <c r="F5" s="11" t="s">
+        <v>2093</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>2094</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>2095</v>
+      </c>
+      <c r="I5" s="11" t="s">
         <v>2096</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>2097</v>
-      </c>
-      <c r="H5" s="11" t="s">
-        <v>2098</v>
-      </c>
-      <c r="I5" s="11" t="s">
-        <v>2099</v>
       </c>
       <c r="J5" s="11" t="s">
         <v>2022</v>
       </c>
       <c r="K5" s="11" t="s">
-        <v>2100</v>
+        <v>2097</v>
       </c>
       <c r="L5" s="11" t="s">
-        <v>2101</v>
+        <v>2098</v>
       </c>
       <c r="M5" s="11" t="s">
         <v>2026</v>
@@ -34941,10 +34941,10 @@
         <v>2025</v>
       </c>
       <c r="P5" s="11" t="s">
-        <v>2102</v>
+        <v>2099</v>
       </c>
       <c r="Q5" s="11" t="s">
-        <v>2103</v>
+        <v>2100</v>
       </c>
       <c r="R5" s="11"/>
       <c r="S5" s="11"/>
@@ -34970,19 +34970,19 @@
         <v>1</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>2101</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>2102</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>2103</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>2104</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="F6" s="4" t="s">
         <v>2105</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>2106</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>2107</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>2108</v>
       </c>
       <c r="G6" s="4">
         <v>85</v>
@@ -35000,16 +35000,16 @@
         <v>1560</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>2109</v>
+        <v>2106</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>2037</v>
+        <v>2039</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>2038</v>
+        <v>2040</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>2110</v>
+        <v>2107</v>
       </c>
       <c r="P6" s="4" t="s">
         <v>2029</v>
@@ -35041,19 +35041,19 @@
         <v>2</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>2108</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>2109</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>2110</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>2111</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="F7" s="6" t="s">
         <v>2112</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>2113</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>2114</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>2060</v>
       </c>
       <c r="G7" s="6">
         <v>90</v>
@@ -35071,16 +35071,16 @@
         <v>546</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>2115</v>
+        <v>2113</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>2037</v>
+        <v>2039</v>
       </c>
       <c r="N7" s="6" t="s">
-        <v>2038</v>
+        <v>2040</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>2116</v>
+        <v>2114</v>
       </c>
       <c r="P7" s="6" t="s">
         <v>2029</v>
@@ -35112,19 +35112,19 @@
         <v>3</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>2115</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>2116</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>2117</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>2118</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>2119</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>2120</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>2121</v>
       </c>
       <c r="G8" s="4">
         <v>82</v>
@@ -35142,16 +35142,16 @@
         <v>1560</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>2122</v>
+        <v>2120</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>2037</v>
+        <v>2039</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>2038</v>
+        <v>2040</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>2123</v>
+        <v>2121</v>
       </c>
       <c r="P8" s="4" t="s">
         <v>2029</v>
@@ -35183,19 +35183,19 @@
         <v>4</v>
       </c>
       <c r="B9" s="6" t="s">
+        <v>2122</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>2123</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>2124</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>2125</v>
       </c>
-      <c r="D9" s="6" t="s">
-        <v>2126</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>2127</v>
-      </c>
       <c r="F9" s="6" t="s">
-        <v>2072</v>
+        <v>2068</v>
       </c>
       <c r="G9" s="6">
         <v>78</v>
@@ -35213,16 +35213,16 @@
         <v>1560</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>2128</v>
+        <v>2126</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>2037</v>
+        <v>2039</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>2038</v>
+        <v>2040</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>2129</v>
+        <v>2127</v>
       </c>
       <c r="P9" s="6" t="s">
         <v>2029</v>
@@ -35254,19 +35254,19 @@
         <v>5</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>2128</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>2129</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>2130</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="E10" s="4" t="s">
         <v>2131</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="F10" s="4" t="s">
         <v>2132</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>2133</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>2028</v>
       </c>
       <c r="G10" s="4">
         <v>70</v>
@@ -35284,16 +35284,16 @@
         <v>1635</v>
       </c>
       <c r="L10" s="4" t="s">
+        <v>2133</v>
+      </c>
+      <c r="M10" s="4" t="s">
+        <v>2039</v>
+      </c>
+      <c r="N10" s="4" t="s">
+        <v>2040</v>
+      </c>
+      <c r="O10" s="4" t="s">
         <v>2134</v>
-      </c>
-      <c r="M10" s="4" t="s">
-        <v>2037</v>
-      </c>
-      <c r="N10" s="4" t="s">
-        <v>2038</v>
-      </c>
-      <c r="O10" s="4" t="s">
-        <v>2135</v>
       </c>
       <c r="P10" s="4" t="s">
         <v>2029</v>
@@ -35325,19 +35325,19 @@
         <v>6</v>
       </c>
       <c r="B11" s="6" t="s">
+        <v>2135</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>2129</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>2136</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>2131</v>
-      </c>
-      <c r="D11" s="6" t="s">
+      <c r="E11" s="6" t="s">
         <v>2137</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="F11" s="6" t="s">
         <v>2138</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>2044</v>
       </c>
       <c r="G11" s="6">
         <v>70</v>
@@ -35358,10 +35358,10 @@
         <v>2139</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>2037</v>
+        <v>2039</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>2038</v>
+        <v>2040</v>
       </c>
       <c r="O11" s="6" t="s">
         <v>2140</v>

</xml_diff>